<commit_message>
update NHL standings, IFHL spreadsheets, and matchday quote templates
</commit_message>
<xml_diff>
--- a/_Classifica IFHL.xlsx
+++ b/_Classifica IFHL.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="26">
   <si>
     <t>GAME 1 of 32</t>
   </si>
@@ -37,19 +37,16 @@
     <t>Beaver Conference</t>
   </si>
   <si>
+    <t>2. Toronto Sasquatch</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
     <t>1. Niagara Falls Goats</t>
   </si>
   <si>
-    <t>W2</t>
-  </si>
-  <si>
-    <t>2. Toronto Sasquatch</t>
-  </si>
-  <si>
     <t>3. Philadelphia Alleghers</t>
-  </si>
-  <si>
-    <t>W1</t>
   </si>
   <si>
     <t>4. Quebec Mooses</t>
@@ -59,9 +56,6 @@
   </si>
   <si>
     <t>6. Montreal Natives</t>
-  </si>
-  <si>
-    <t>L1</t>
   </si>
   <si>
     <t>7. Halifax Lumberjacks</t>
@@ -92,9 +86,6 @@
   </si>
   <si>
     <t>7. Pittsburgh Bagpipes</t>
-  </si>
-  <si>
-    <t>L2</t>
   </si>
   <si>
     <t>8. Las Vegas Jackpots</t>
@@ -364,7 +355,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="25.75"/>
-    <col customWidth="1" min="2" max="2" width="12.0"/>
+    <col customWidth="1" min="2" max="2" width="13.13"/>
     <col customWidth="1" min="3" max="3" width="3.63"/>
     <col customWidth="1" min="4" max="4" width="3.0"/>
     <col customWidth="1" min="5" max="5" width="3.5"/>
@@ -476,10 +467,10 @@
         <v>8</v>
       </c>
       <c r="B4" s="1">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="C4" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="D4" s="1">
         <v>0.0</v>
@@ -491,9 +482,9 @@
         <v>9</v>
       </c>
       <c r="G4" s="3">
-        <v>100.99</v>
+        <v>0.0</v>
       </c>
-      <c r="H4" s="4"/>
+      <c r="H4" s="1"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -518,10 +509,10 @@
         <v>10</v>
       </c>
       <c r="B5" s="1">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="C5" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="D5" s="1">
         <v>0.0</v>
@@ -533,9 +524,9 @@
         <v>9</v>
       </c>
       <c r="G5" s="3">
-        <v>137.11</v>
+        <v>0.0</v>
       </c>
-      <c r="H5" s="1"/>
+      <c r="H5" s="4"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
@@ -560,22 +551,22 @@
         <v>11</v>
       </c>
       <c r="B6" s="1">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="C6" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D6" s="1">
         <v>0.0</v>
       </c>
       <c r="E6" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G6" s="3">
-        <v>136.2</v>
+        <v>0.0</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -599,25 +590,25 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="C7" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D7" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E7" s="1">
         <v>0.0</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G7" s="3">
-        <v>111.1</v>
+        <v>0.0</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -641,25 +632,25 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="C8" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D8" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E8" s="1">
         <v>0.0</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G8" s="3">
-        <v>113.36</v>
+        <v>0.0</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -683,25 +674,25 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="C9" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D9" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E9" s="1">
         <v>0.0</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G9" s="3">
-        <v>90.19</v>
+        <v>0.0</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -725,25 +716,25 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B10" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="C10" s="1">
         <v>0.0</v>
       </c>
       <c r="D10" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E10" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G10" s="3">
-        <v>110.18</v>
+        <v>0.0</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
@@ -767,25 +758,25 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B11" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="C11" s="1">
         <v>0.0</v>
       </c>
       <c r="D11" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E11" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G11" s="3">
-        <v>78.97</v>
+        <v>0.0</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -837,7 +828,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -867,13 +858,13 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B14" s="1">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="C14" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="D14" s="1">
         <v>0.0</v>
@@ -885,7 +876,7 @@
         <v>9</v>
       </c>
       <c r="G14" s="3">
-        <v>125.07</v>
+        <v>0.0</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -909,13 +900,13 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B15" s="1">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="C15" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="D15" s="1">
         <v>0.0</v>
@@ -927,7 +918,7 @@
         <v>9</v>
       </c>
       <c r="G15" s="3">
-        <v>124.94</v>
+        <v>0.0</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -951,25 +942,25 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B16" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="C16" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D16" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E16" s="1">
         <v>0.0</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G16" s="3">
-        <v>94.79</v>
+        <v>0.0</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -993,25 +984,25 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B17" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="C17" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D17" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E17" s="1">
         <v>0.0</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G17" s="3">
-        <v>94.29</v>
+        <v>0.0</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
@@ -1035,25 +1026,25 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B18" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="C18" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D18" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E18" s="1">
         <v>0.0</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G18" s="3">
-        <v>77.47</v>
+        <v>0.0</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -1077,25 +1068,25 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="1">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="C19" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D19" s="1">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E19" s="1">
         <v>0.0</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G19" s="3">
-        <v>69.05</v>
+        <v>0.0</v>
       </c>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
@@ -1119,7 +1110,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20" s="1">
         <v>0.0</v>
@@ -1134,10 +1125,10 @@
         <v>0.0</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="G20" s="3">
-        <v>78.36</v>
+        <v>0.0</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -1161,7 +1152,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B21" s="1">
         <v>0.0</v>
@@ -1176,10 +1167,10 @@
         <v>0.0</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="G21" s="3">
-        <v>65.31</v>
+        <v>0.0</v>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>

</xml_diff>